<commit_message>
Lecture 16 to 27 Added
</commit_message>
<xml_diff>
--- a/MS Excel Crash Course/Lecture 11.xlsx
+++ b/MS Excel Crash Course/Lecture 11.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AR Boot Camp 2k26\MS Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AR Boot Camp 2k26\MS Excel Crash Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13EF9F99-C076-43A0-93CB-827C9A20CD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38F2A84-2A3A-4EBA-B533-7C7ED49C57AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-10409]h:mm:ss\ am/pm;@"/>
+    <numFmt numFmtId="164" formatCode="[$-10409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -161,10 +161,7 @@
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -174,6 +171,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -465,26 +465,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>0</v>
       </c>
     </row>
@@ -545,18 +545,18 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>